<commit_message>
Added some annotations for calculations to be made
</commit_message>
<xml_diff>
--- a/Yield/RES_field_datasheet_jdx.xlsx
+++ b/Yield/RES_field_datasheet_jdx.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhangdakui/Documents/GitHub/ERW/Yield/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zhang\Documents\GitHub\ERW\Yield\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB96D3AC-257A-984E-B1A4-C4B4775137FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{7065DB47-097C-C04F-ADEF-4C289C6D55B0}"/>
+    <workbookView xWindow="0" yWindow="765" windowWidth="30240" windowHeight="18885"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>Plot</t>
   </si>
@@ -102,13 +101,37 @@
   </si>
   <si>
     <t>OD_Straw_g</t>
+  </si>
+  <si>
+    <t>Paper+Grains+Rubber_Band</t>
+  </si>
+  <si>
+    <t>(5xpaperbag+5Rubberband)/5</t>
+  </si>
+  <si>
+    <t>D=B-C</t>
+  </si>
+  <si>
+    <t>F=D-E</t>
+  </si>
+  <si>
+    <t>E=</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>HI=E/D</t>
+  </si>
+  <si>
+    <t>Usually around 0.51</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -472,17 +495,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF552B86-4BA9-0C49-BA29-956140839636}">
-  <dimension ref="A1:G16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H21"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="26.6640625" customWidth="1"/>
-    <col min="3" max="3" width="12.1640625" customWidth="1"/>
+    <col min="3" max="3" width="12.109375" customWidth="1"/>
     <col min="4" max="4" width="18.6640625" customWidth="1"/>
     <col min="5" max="5" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -505,7 +528,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -516,7 +539,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -527,7 +550,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -538,7 +561,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -549,7 +572,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -560,7 +583,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -571,7 +594,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -582,7 +605,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -593,7 +616,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -604,7 +627,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -615,7 +638,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -626,7 +649,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7">
       <c r="A13" t="s">
         <v>6</v>
       </c>
@@ -637,7 +660,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -648,7 +671,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7">
       <c r="A15" t="s">
         <v>7</v>
       </c>
@@ -659,7 +682,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -668,6 +691,38 @@
       </c>
       <c r="C16">
         <v>120</v>
+      </c>
+    </row>
+    <row r="18" spans="4:8">
+      <c r="D18" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="4:8">
+      <c r="D19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="4:8">
+      <c r="D20" t="s">
+        <v>26</v>
+      </c>
+      <c r="E20" t="s">
+        <v>22</v>
+      </c>
+      <c r="G20" t="s">
+        <v>27</v>
+      </c>
+      <c r="H20" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="21" spans="4:8">
+      <c r="D21" t="s">
+        <v>28</v>
+      </c>
+      <c r="E21" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>